<commit_message>
docs: agregar columna Estado y cambiar frecuencia a Diaria en metadatos C360
- Metadatos Tabla: nueva columna 'Estado' = Activo para las 12 tablas;
  frecuencia de actualización cambiada de Semanal a Diaria
- Metadatos Columna: nueva columna 'Estado' = Activo para las 154 columnas

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CcS2rRicqWu6BQakKjvAJK
</commit_message>
<xml_diff>
--- a/11_Metadatos_Cliente360.xlsx
+++ b/11_Metadatos_Cliente360.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,6 +52,10 @@
     <font>
       <name val="Arial"/>
       <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -109,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -123,6 +127,12 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -600,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S13"/>
+  <dimension ref="A1:T13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -717,6 +727,11 @@
       </c>
       <c r="S1" s="6" t="inlineStr">
         <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="T1" s="6" t="inlineStr">
+        <is>
           <t>Capa Medallón</t>
         </is>
       </c>
@@ -784,7 +799,7 @@
       </c>
       <c r="M2" s="7" t="inlineStr">
         <is>
-          <t>Semanal</t>
+          <t>Diaria</t>
         </is>
       </c>
       <c r="N2" s="7" t="inlineStr">
@@ -812,7 +827,12 @@
           <t>Contiene datos personales y sensibles de salud. SCD Tipo 1: solo versión vigente.</t>
         </is>
       </c>
-      <c r="S2" s="7" t="inlineStr">
+      <c r="S2" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="T2" s="7" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
@@ -881,7 +901,7 @@
       </c>
       <c r="M3" s="8" t="inlineStr">
         <is>
-          <t>Semanal</t>
+          <t>Diaria</t>
         </is>
       </c>
       <c r="N3" s="8" t="inlineStr">
@@ -909,7 +929,12 @@
           <t>Contiene datos laborales y de contacto del trabajador. SCD Tipo 1: solo versión vigente.</t>
         </is>
       </c>
-      <c r="S3" s="8" t="inlineStr">
+      <c r="S3" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="T3" s="8" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
@@ -978,7 +1003,7 @@
       </c>
       <c r="M4" s="7" t="inlineStr">
         <is>
-          <t>Semanal</t>
+          <t>Diaria</t>
         </is>
       </c>
       <c r="N4" s="7" t="inlineStr">
@@ -1006,7 +1031,12 @@
           <t>Contiene datos de asegurados y beneficiarios. SCD Tipo 1: solo versión vigente.</t>
         </is>
       </c>
-      <c r="S4" s="7" t="inlineStr">
+      <c r="S4" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="T4" s="7" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
@@ -1075,7 +1105,7 @@
       </c>
       <c r="M5" s="8" t="inlineStr">
         <is>
-          <t>Semanal</t>
+          <t>Diaria</t>
         </is>
       </c>
       <c r="N5" s="8" t="inlineStr">
@@ -1103,7 +1133,12 @@
           <t>Tabla maestra del cliente único AXA. SCD Tipo 1: atributo con mayor score de calidad y selección.</t>
         </is>
       </c>
-      <c r="S5" s="8" t="inlineStr">
+      <c r="S5" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="T5" s="8" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
@@ -1172,7 +1207,7 @@
       </c>
       <c r="M6" s="7" t="inlineStr">
         <is>
-          <t>Semanal</t>
+          <t>Diaria</t>
         </is>
       </c>
       <c r="N6" s="7" t="inlineStr">
@@ -1200,7 +1235,12 @@
           <t>Tabla de control; no contiene datos personales. Misma estructura que la del Validador de Calidad.</t>
         </is>
       </c>
-      <c r="S6" s="7" t="inlineStr">
+      <c r="S6" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="T6" s="7" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
@@ -1269,7 +1309,7 @@
       </c>
       <c r="M7" s="8" t="inlineStr">
         <is>
-          <t>Semanal</t>
+          <t>Diaria</t>
         </is>
       </c>
       <c r="N7" s="8" t="inlineStr">
@@ -1297,7 +1337,12 @@
           <t>Catálogo de reglas de selección y transformación. SCD Tipo 2: guarda historial de cambios.</t>
         </is>
       </c>
-      <c r="S7" s="8" t="inlineStr">
+      <c r="S7" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="T7" s="8" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
@@ -1366,7 +1411,7 @@
       </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
-          <t>Semanal</t>
+          <t>Diaria</t>
         </is>
       </c>
       <c r="N8" s="7" t="inlineStr">
@@ -1394,7 +1439,12 @@
           <t>Sin datos personales. Compartida con el Validador de Calidad.</t>
         </is>
       </c>
-      <c r="S8" s="7" t="inlineStr">
+      <c r="S8" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="T8" s="7" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
@@ -1463,7 +1513,7 @@
       </c>
       <c r="M9" s="8" t="inlineStr">
         <is>
-          <t>Semanal</t>
+          <t>Diaria</t>
         </is>
       </c>
       <c r="N9" s="8" t="inlineStr">
@@ -1491,7 +1541,12 @@
           <t>Contiene id_cliente; datos sensibles de atributos marcados sospechosos. SCD Tipo 2.</t>
         </is>
       </c>
-      <c r="S9" s="8" t="inlineStr">
+      <c r="S9" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="T9" s="8" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
@@ -1560,7 +1615,7 @@
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>Semanal</t>
+          <t>Diaria</t>
         </is>
       </c>
       <c r="N10" s="7" t="inlineStr">
@@ -1588,7 +1643,12 @@
           <t>Catálogo de fuentes; no contiene datos personales. SCD Tipo 1.</t>
         </is>
       </c>
-      <c r="S10" s="7" t="inlineStr">
+      <c r="S10" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="T10" s="7" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
@@ -1657,7 +1717,7 @@
       </c>
       <c r="M11" s="8" t="inlineStr">
         <is>
-          <t>Semanal</t>
+          <t>Diaria</t>
         </is>
       </c>
       <c r="N11" s="8" t="inlineStr">
@@ -1685,7 +1745,12 @@
           <t>Contiene referencias a clientes vía fk_fuente_cliente. SCD Tipo 2. Tabla central del modelo analítico.</t>
         </is>
       </c>
-      <c r="S11" s="8" t="inlineStr">
+      <c r="S11" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="T11" s="8" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
@@ -1754,7 +1819,7 @@
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>Semanal</t>
+          <t>Diaria</t>
         </is>
       </c>
       <c r="N12" s="7" t="inlineStr">
@@ -1782,7 +1847,12 @@
           <t>Contiene id_cliente y valores de atributos procesados. SCD Tipo 2.</t>
         </is>
       </c>
-      <c r="S12" s="7" t="inlineStr">
+      <c r="S12" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="T12" s="7" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
@@ -1851,7 +1921,7 @@
       </c>
       <c r="M13" s="8" t="inlineStr">
         <is>
-          <t>Semanal</t>
+          <t>Diaria</t>
         </is>
       </c>
       <c r="N13" s="8" t="inlineStr">
@@ -1879,7 +1949,12 @@
           <t>Vista de consulta; no almacena datos. Filtra marca_sospechoso = 1.</t>
         </is>
       </c>
-      <c r="S13" s="8" t="inlineStr">
+      <c r="S13" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="T13" s="8" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
@@ -1896,7 +1971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N155"/>
+  <dimension ref="A1:O155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1913,6 +1988,7 @@
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="35" customWidth="1" min="13" max="13"/>
     <col width="45" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
@@ -1986,6 +2062,11 @@
           <t>Observaciones</t>
         </is>
       </c>
+      <c r="O1" s="6" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="35" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
@@ -2050,6 +2131,11 @@
         </is>
       </c>
       <c r="N2" s="7" t="inlineStr"/>
+      <c r="O2" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="35" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
@@ -2114,6 +2200,11 @@
           <t>Homologado según tabla de parámetros dim_parametros</t>
         </is>
       </c>
+      <c r="O3" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="35" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
@@ -2174,6 +2265,11 @@
         </is>
       </c>
       <c r="N4" s="7" t="inlineStr"/>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="35" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
@@ -2234,6 +2330,11 @@
         </is>
       </c>
       <c r="N5" s="8" t="inlineStr"/>
+      <c r="O5" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="35" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
@@ -2294,6 +2395,11 @@
         </is>
       </c>
       <c r="N6" s="7" t="inlineStr"/>
+      <c r="O6" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="35" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
@@ -2354,6 +2460,11 @@
         </is>
       </c>
       <c r="N7" s="8" t="inlineStr"/>
+      <c r="O7" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="35" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -2414,6 +2525,11 @@
         </is>
       </c>
       <c r="N8" s="7" t="inlineStr"/>
+      <c r="O8" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="35" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
@@ -2474,6 +2590,11 @@
         </is>
       </c>
       <c r="N9" s="8" t="inlineStr"/>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="35" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -2538,6 +2659,11 @@
           <t>Homologado según dim_parametros</t>
         </is>
       </c>
+      <c r="O10" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="35" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
@@ -2598,6 +2724,11 @@
         </is>
       </c>
       <c r="N11" s="8" t="inlineStr"/>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="35" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
@@ -2658,6 +2789,11 @@
         </is>
       </c>
       <c r="N12" s="7" t="inlineStr"/>
+      <c r="O12" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="35" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
@@ -2718,6 +2854,11 @@
         </is>
       </c>
       <c r="N13" s="8" t="inlineStr"/>
+      <c r="O13" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="35" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
@@ -2782,6 +2923,11 @@
           <t>Homologado: Activo / No Activo</t>
         </is>
       </c>
+      <c r="O14" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="35" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
@@ -2842,6 +2988,11 @@
         </is>
       </c>
       <c r="N15" s="8" t="inlineStr"/>
+      <c r="O15" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="35" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
@@ -2902,6 +3053,11 @@
         </is>
       </c>
       <c r="N16" s="7" t="inlineStr"/>
+      <c r="O16" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="35" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
@@ -2962,6 +3118,11 @@
         </is>
       </c>
       <c r="N17" s="8" t="inlineStr"/>
+      <c r="O17" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="35" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
@@ -3022,6 +3183,11 @@
         </is>
       </c>
       <c r="N18" s="7" t="inlineStr"/>
+      <c r="O18" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="35" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
@@ -3086,6 +3252,11 @@
           <t>Valor fijo: core_bh</t>
         </is>
       </c>
+      <c r="O19" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="35" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
@@ -3150,6 +3321,11 @@
         </is>
       </c>
       <c r="N20" s="7" t="inlineStr"/>
+      <c r="O20" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="35" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
@@ -3214,6 +3390,11 @@
         </is>
       </c>
       <c r="N21" s="8" t="inlineStr"/>
+      <c r="O21" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="35" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
@@ -3278,6 +3459,11 @@
           <t>Homologado según dim_parametros</t>
         </is>
       </c>
+      <c r="O22" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="35" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
@@ -3338,6 +3524,11 @@
         </is>
       </c>
       <c r="N23" s="8" t="inlineStr"/>
+      <c r="O23" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="35" customHeight="1">
       <c r="A24" s="7" t="inlineStr">
@@ -3398,6 +3589,11 @@
         </is>
       </c>
       <c r="N24" s="7" t="inlineStr"/>
+      <c r="O24" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="35" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
@@ -3458,6 +3654,11 @@
         </is>
       </c>
       <c r="N25" s="8" t="inlineStr"/>
+      <c r="O25" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="35" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
@@ -3518,6 +3719,11 @@
         </is>
       </c>
       <c r="N26" s="7" t="inlineStr"/>
+      <c r="O26" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="35" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
@@ -3578,6 +3784,11 @@
         </is>
       </c>
       <c r="N27" s="8" t="inlineStr"/>
+      <c r="O27" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="35" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
@@ -3638,6 +3849,11 @@
         </is>
       </c>
       <c r="N28" s="7" t="inlineStr"/>
+      <c r="O28" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="35" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
@@ -3698,6 +3914,11 @@
         </is>
       </c>
       <c r="N29" s="8" t="inlineStr"/>
+      <c r="O29" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="35" customHeight="1">
       <c r="A30" s="7" t="inlineStr">
@@ -3758,6 +3979,11 @@
         </is>
       </c>
       <c r="N30" s="7" t="inlineStr"/>
+      <c r="O30" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="35" customHeight="1">
       <c r="A31" s="8" t="inlineStr">
@@ -3818,6 +4044,11 @@
         </is>
       </c>
       <c r="N31" s="8" t="inlineStr"/>
+      <c r="O31" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="35" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
@@ -3878,6 +4109,11 @@
         </is>
       </c>
       <c r="N32" s="7" t="inlineStr"/>
+      <c r="O32" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="35" customHeight="1">
       <c r="A33" s="8" t="inlineStr">
@@ -3938,6 +4174,11 @@
         </is>
       </c>
       <c r="N33" s="8" t="inlineStr"/>
+      <c r="O33" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="35" customHeight="1">
       <c r="A34" s="7" t="inlineStr">
@@ -3998,6 +4239,11 @@
         </is>
       </c>
       <c r="N34" s="7" t="inlineStr"/>
+      <c r="O34" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="35" customHeight="1">
       <c r="A35" s="8" t="inlineStr">
@@ -4058,6 +4304,11 @@
         </is>
       </c>
       <c r="N35" s="8" t="inlineStr"/>
+      <c r="O35" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="35" customHeight="1">
       <c r="A36" s="7" t="inlineStr">
@@ -4122,6 +4373,11 @@
           <t>Valor fijo: core_as400</t>
         </is>
       </c>
+      <c r="O36" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="35" customHeight="1">
       <c r="A37" s="8" t="inlineStr">
@@ -4186,6 +4442,11 @@
         </is>
       </c>
       <c r="N37" s="8" t="inlineStr"/>
+      <c r="O37" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="35" customHeight="1">
       <c r="A38" s="7" t="inlineStr">
@@ -4250,6 +4511,11 @@
         </is>
       </c>
       <c r="N38" s="7" t="inlineStr"/>
+      <c r="O38" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="35" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
@@ -4314,6 +4580,11 @@
           <t>Homologado según dim_parametros</t>
         </is>
       </c>
+      <c r="O39" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="35" customHeight="1">
       <c r="A40" s="7" t="inlineStr">
@@ -4374,6 +4645,11 @@
         </is>
       </c>
       <c r="N40" s="7" t="inlineStr"/>
+      <c r="O40" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="35" customHeight="1">
       <c r="A41" s="8" t="inlineStr">
@@ -4434,6 +4710,11 @@
         </is>
       </c>
       <c r="N41" s="8" t="inlineStr"/>
+      <c r="O41" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="35" customHeight="1">
       <c r="A42" s="7" t="inlineStr">
@@ -4494,6 +4775,11 @@
         </is>
       </c>
       <c r="N42" s="7" t="inlineStr"/>
+      <c r="O42" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="35" customHeight="1">
       <c r="A43" s="8" t="inlineStr">
@@ -4554,6 +4840,11 @@
         </is>
       </c>
       <c r="N43" s="8" t="inlineStr"/>
+      <c r="O43" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="35" customHeight="1">
       <c r="A44" s="7" t="inlineStr">
@@ -4614,6 +4905,11 @@
         </is>
       </c>
       <c r="N44" s="7" t="inlineStr"/>
+      <c r="O44" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="35" customHeight="1">
       <c r="A45" s="8" t="inlineStr">
@@ -4674,6 +4970,11 @@
         </is>
       </c>
       <c r="N45" s="8" t="inlineStr"/>
+      <c r="O45" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="35" customHeight="1">
       <c r="A46" s="7" t="inlineStr">
@@ -4734,6 +5035,11 @@
         </is>
       </c>
       <c r="N46" s="7" t="inlineStr"/>
+      <c r="O46" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="35" customHeight="1">
       <c r="A47" s="8" t="inlineStr">
@@ -4794,6 +5100,11 @@
         </is>
       </c>
       <c r="N47" s="8" t="inlineStr"/>
+      <c r="O47" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="35" customHeight="1">
       <c r="A48" s="7" t="inlineStr">
@@ -4854,6 +5165,11 @@
         </is>
       </c>
       <c r="N48" s="7" t="inlineStr"/>
+      <c r="O48" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="35" customHeight="1">
       <c r="A49" s="8" t="inlineStr">
@@ -4914,6 +5230,11 @@
         </is>
       </c>
       <c r="N49" s="8" t="inlineStr"/>
+      <c r="O49" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="35" customHeight="1">
       <c r="A50" s="7" t="inlineStr">
@@ -4978,6 +5299,11 @@
           <t>Valores: Soltero, Casado, Divorciado, Viudo, Unión Libre, etc.</t>
         </is>
       </c>
+      <c r="O50" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="35" customHeight="1">
       <c r="A51" s="8" t="inlineStr">
@@ -5038,6 +5364,11 @@
         </is>
       </c>
       <c r="N51" s="8" t="inlineStr"/>
+      <c r="O51" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="35" customHeight="1">
       <c r="A52" s="7" t="inlineStr">
@@ -5102,6 +5433,11 @@
           <t>Valor fijo: core_sise</t>
         </is>
       </c>
+      <c r="O52" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="35" customHeight="1">
       <c r="A53" s="8" t="inlineStr">
@@ -5166,6 +5502,11 @@
         </is>
       </c>
       <c r="N53" s="8" t="inlineStr"/>
+      <c r="O53" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="35" customHeight="1">
       <c r="A54" s="7" t="inlineStr">
@@ -5230,6 +5571,11 @@
         </is>
       </c>
       <c r="N54" s="7" t="inlineStr"/>
+      <c r="O54" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="35" customHeight="1">
       <c r="A55" s="8" t="inlineStr">
@@ -5290,6 +5636,11 @@
         </is>
       </c>
       <c r="N55" s="8" t="inlineStr"/>
+      <c r="O55" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="35" customHeight="1">
       <c r="A56" s="7" t="inlineStr">
@@ -5350,6 +5701,11 @@
         </is>
       </c>
       <c r="N56" s="7" t="inlineStr"/>
+      <c r="O56" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="35" customHeight="1">
       <c r="A57" s="8" t="inlineStr">
@@ -5410,6 +5766,11 @@
         </is>
       </c>
       <c r="N57" s="8" t="inlineStr"/>
+      <c r="O57" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="35" customHeight="1">
       <c r="A58" s="7" t="inlineStr">
@@ -5470,6 +5831,11 @@
         </is>
       </c>
       <c r="N58" s="7" t="inlineStr"/>
+      <c r="O58" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="35" customHeight="1">
       <c r="A59" s="8" t="inlineStr">
@@ -5530,6 +5896,11 @@
         </is>
       </c>
       <c r="N59" s="8" t="inlineStr"/>
+      <c r="O59" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="35" customHeight="1">
       <c r="A60" s="7" t="inlineStr">
@@ -5590,6 +5961,11 @@
         </is>
       </c>
       <c r="N60" s="7" t="inlineStr"/>
+      <c r="O60" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="35" customHeight="1">
       <c r="A61" s="8" t="inlineStr">
@@ -5650,6 +6026,11 @@
         </is>
       </c>
       <c r="N61" s="8" t="inlineStr"/>
+      <c r="O61" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="35" customHeight="1">
       <c r="A62" s="7" t="inlineStr">
@@ -5710,6 +6091,11 @@
         </is>
       </c>
       <c r="N62" s="7" t="inlineStr"/>
+      <c r="O62" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="35" customHeight="1">
       <c r="A63" s="8" t="inlineStr">
@@ -5770,6 +6156,11 @@
         </is>
       </c>
       <c r="N63" s="8" t="inlineStr"/>
+      <c r="O63" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="35" customHeight="1">
       <c r="A64" s="7" t="inlineStr">
@@ -5830,6 +6221,11 @@
         </is>
       </c>
       <c r="N64" s="7" t="inlineStr"/>
+      <c r="O64" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="35" customHeight="1">
       <c r="A65" s="8" t="inlineStr">
@@ -5890,6 +6286,11 @@
         </is>
       </c>
       <c r="N65" s="8" t="inlineStr"/>
+      <c r="O65" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="35" customHeight="1">
       <c r="A66" s="7" t="inlineStr">
@@ -5950,6 +6351,11 @@
         </is>
       </c>
       <c r="N66" s="7" t="inlineStr"/>
+      <c r="O66" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="35" customHeight="1">
       <c r="A67" s="8" t="inlineStr">
@@ -6010,6 +6416,11 @@
         </is>
       </c>
       <c r="N67" s="8" t="inlineStr"/>
+      <c r="O67" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="35" customHeight="1">
       <c r="A68" s="7" t="inlineStr">
@@ -6070,6 +6481,11 @@
         </is>
       </c>
       <c r="N68" s="7" t="inlineStr"/>
+      <c r="O68" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="35" customHeight="1">
       <c r="A69" s="8" t="inlineStr">
@@ -6130,6 +6546,11 @@
         </is>
       </c>
       <c r="N69" s="8" t="inlineStr"/>
+      <c r="O69" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="35" customHeight="1">
       <c r="A70" s="7" t="inlineStr">
@@ -6190,6 +6611,11 @@
         </is>
       </c>
       <c r="N70" s="7" t="inlineStr"/>
+      <c r="O70" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="35" customHeight="1">
       <c r="A71" s="8" t="inlineStr">
@@ -6254,6 +6680,11 @@
         </is>
       </c>
       <c r="N71" s="8" t="inlineStr"/>
+      <c r="O71" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="35" customHeight="1">
       <c r="A72" s="7" t="inlineStr">
@@ -6318,6 +6749,11 @@
         </is>
       </c>
       <c r="N72" s="7" t="inlineStr"/>
+      <c r="O72" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="35" customHeight="1">
       <c r="A73" s="8" t="inlineStr">
@@ -6378,6 +6814,11 @@
         </is>
       </c>
       <c r="N73" s="8" t="inlineStr"/>
+      <c r="O73" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="35" customHeight="1">
       <c r="A74" s="7" t="inlineStr">
@@ -6438,6 +6879,11 @@
         </is>
       </c>
       <c r="N74" s="7" t="inlineStr"/>
+      <c r="O74" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="35" customHeight="1">
       <c r="A75" s="8" t="inlineStr">
@@ -6498,6 +6944,11 @@
         </is>
       </c>
       <c r="N75" s="8" t="inlineStr"/>
+      <c r="O75" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="35" customHeight="1">
       <c r="A76" s="7" t="inlineStr">
@@ -6558,6 +7009,11 @@
         </is>
       </c>
       <c r="N76" s="7" t="inlineStr"/>
+      <c r="O76" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="35" customHeight="1">
       <c r="A77" s="8" t="inlineStr">
@@ -6618,6 +7074,11 @@
         </is>
       </c>
       <c r="N77" s="8" t="inlineStr"/>
+      <c r="O77" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="35" customHeight="1">
       <c r="A78" s="7" t="inlineStr">
@@ -6678,6 +7139,11 @@
         </is>
       </c>
       <c r="N78" s="7" t="inlineStr"/>
+      <c r="O78" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="35" customHeight="1">
       <c r="A79" s="8" t="inlineStr">
@@ -6738,6 +7204,11 @@
         </is>
       </c>
       <c r="N79" s="8" t="inlineStr"/>
+      <c r="O79" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="35" customHeight="1">
       <c r="A80" s="7" t="inlineStr">
@@ -6798,6 +7269,11 @@
         </is>
       </c>
       <c r="N80" s="7" t="inlineStr"/>
+      <c r="O80" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="35" customHeight="1">
       <c r="A81" s="8" t="inlineStr">
@@ -6858,6 +7334,11 @@
         </is>
       </c>
       <c r="N81" s="8" t="inlineStr"/>
+      <c r="O81" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="35" customHeight="1">
       <c r="A82" s="7" t="inlineStr">
@@ -6922,6 +7403,11 @@
         </is>
       </c>
       <c r="N82" s="7" t="inlineStr"/>
+      <c r="O82" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="35" customHeight="1">
       <c r="A83" s="8" t="inlineStr">
@@ -6986,6 +7472,11 @@
         </is>
       </c>
       <c r="N83" s="8" t="inlineStr"/>
+      <c r="O83" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="35" customHeight="1">
       <c r="A84" s="7" t="inlineStr">
@@ -7050,6 +7541,11 @@
         </is>
       </c>
       <c r="N84" s="7" t="inlineStr"/>
+      <c r="O84" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="35" customHeight="1">
       <c r="A85" s="8" t="inlineStr">
@@ -7110,6 +7606,11 @@
         </is>
       </c>
       <c r="N85" s="8" t="inlineStr"/>
+      <c r="O85" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="35" customHeight="1">
       <c r="A86" s="7" t="inlineStr">
@@ -7174,6 +7675,11 @@
           <t>Formato: catalogo.esquema.tabla.atributo</t>
         </is>
       </c>
+      <c r="O86" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="35" customHeight="1">
       <c r="A87" s="8" t="inlineStr">
@@ -7238,6 +7744,11 @@
           <t>Valores: seleccion, transformacion</t>
         </is>
       </c>
+      <c r="O87" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="35" customHeight="1">
       <c r="A88" s="7" t="inlineStr">
@@ -7298,6 +7809,11 @@
         </is>
       </c>
       <c r="N88" s="7" t="inlineStr"/>
+      <c r="O88" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="35" customHeight="1">
       <c r="A89" s="8" t="inlineStr">
@@ -7358,6 +7874,11 @@
         </is>
       </c>
       <c r="N89" s="8" t="inlineStr"/>
+      <c r="O89" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="35" customHeight="1">
       <c r="A90" s="7" t="inlineStr">
@@ -7418,6 +7939,11 @@
         </is>
       </c>
       <c r="N90" s="7" t="inlineStr"/>
+      <c r="O90" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="35" customHeight="1">
       <c r="A91" s="8" t="inlineStr">
@@ -7478,6 +8004,11 @@
         </is>
       </c>
       <c r="N91" s="8" t="inlineStr"/>
+      <c r="O91" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="35" customHeight="1">
       <c r="A92" s="7" t="inlineStr">
@@ -7542,6 +8073,11 @@
         </is>
       </c>
       <c r="N92" s="7" t="inlineStr"/>
+      <c r="O92" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="35" customHeight="1">
       <c r="A93" s="8" t="inlineStr">
@@ -7610,6 +8146,11 @@
           <t>NULL = registro vigente activo</t>
         </is>
       </c>
+      <c r="O93" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="35" customHeight="1">
       <c r="A94" s="7" t="inlineStr">
@@ -7674,6 +8215,11 @@
         </is>
       </c>
       <c r="N94" s="7" t="inlineStr"/>
+      <c r="O94" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="35" customHeight="1">
       <c r="A95" s="8" t="inlineStr">
@@ -7738,6 +8284,11 @@
         </is>
       </c>
       <c r="N95" s="8" t="inlineStr"/>
+      <c r="O95" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="35" customHeight="1">
       <c r="A96" s="7" t="inlineStr">
@@ -7802,6 +8353,11 @@
         </is>
       </c>
       <c r="N96" s="7" t="inlineStr"/>
+      <c r="O96" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="35" customHeight="1">
       <c r="A97" s="8" t="inlineStr">
@@ -7862,6 +8418,11 @@
         </is>
       </c>
       <c r="N97" s="8" t="inlineStr"/>
+      <c r="O97" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="35" customHeight="1">
       <c r="A98" s="7" t="inlineStr">
@@ -7922,6 +8483,11 @@
         </is>
       </c>
       <c r="N98" s="7" t="inlineStr"/>
+      <c r="O98" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="35" customHeight="1">
       <c r="A99" s="8" t="inlineStr">
@@ -7982,6 +8548,11 @@
         </is>
       </c>
       <c r="N99" s="8" t="inlineStr"/>
+      <c r="O99" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="35" customHeight="1">
       <c r="A100" s="7" t="inlineStr">
@@ -8042,6 +8613,11 @@
         </is>
       </c>
       <c r="N100" s="7" t="inlineStr"/>
+      <c r="O100" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="35" customHeight="1">
       <c r="A101" s="8" t="inlineStr">
@@ -8102,6 +8678,11 @@
         </is>
       </c>
       <c r="N101" s="8" t="inlineStr"/>
+      <c r="O101" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="35" customHeight="1">
       <c r="A102" s="7" t="inlineStr">
@@ -8162,6 +8743,11 @@
         </is>
       </c>
       <c r="N102" s="7" t="inlineStr"/>
+      <c r="O102" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="35" customHeight="1">
       <c r="A103" s="8" t="inlineStr">
@@ -8222,6 +8808,11 @@
         </is>
       </c>
       <c r="N103" s="8" t="inlineStr"/>
+      <c r="O103" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="35" customHeight="1">
       <c r="A104" s="7" t="inlineStr">
@@ -8282,6 +8873,11 @@
         </is>
       </c>
       <c r="N104" s="7" t="inlineStr"/>
+      <c r="O104" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="35" customHeight="1">
       <c r="A105" s="8" t="inlineStr">
@@ -8346,6 +8942,11 @@
           <t>Valores: 0 = día hábil, 1 = fin de semana</t>
         </is>
       </c>
+      <c r="O105" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="35" customHeight="1">
       <c r="A106" s="7" t="inlineStr">
@@ -8410,6 +9011,11 @@
         </is>
       </c>
       <c r="N106" s="7" t="inlineStr"/>
+      <c r="O106" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="35" customHeight="1">
       <c r="A107" s="8" t="inlineStr">
@@ -8474,6 +9080,11 @@
         </is>
       </c>
       <c r="N107" s="8" t="inlineStr"/>
+      <c r="O107" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="35" customHeight="1">
       <c r="A108" s="7" t="inlineStr">
@@ -8534,6 +9145,11 @@
         </is>
       </c>
       <c r="N108" s="7" t="inlineStr"/>
+      <c r="O108" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="35" customHeight="1">
       <c r="A109" s="8" t="inlineStr">
@@ -8594,6 +9210,11 @@
         </is>
       </c>
       <c r="N109" s="8" t="inlineStr"/>
+      <c r="O109" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="35" customHeight="1">
       <c r="A110" s="7" t="inlineStr">
@@ -8654,6 +9275,11 @@
         </is>
       </c>
       <c r="N110" s="7" t="inlineStr"/>
+      <c r="O110" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="35" customHeight="1">
       <c r="A111" s="8" t="inlineStr">
@@ -8718,6 +9344,11 @@
           <t>Valores: 1 = sospechoso, 0 = no sospechoso</t>
         </is>
       </c>
+      <c r="O111" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="35" customHeight="1">
       <c r="A112" s="7" t="inlineStr">
@@ -8782,6 +9413,11 @@
         </is>
       </c>
       <c r="N112" s="7" t="inlineStr"/>
+      <c r="O112" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="35" customHeight="1">
       <c r="A113" s="8" t="inlineStr">
@@ -8846,6 +9482,11 @@
         </is>
       </c>
       <c r="N113" s="8" t="inlineStr"/>
+      <c r="O113" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="35" customHeight="1">
       <c r="A114" s="7" t="inlineStr">
@@ -8914,6 +9555,11 @@
           <t>NULL = registro vigente</t>
         </is>
       </c>
+      <c r="O114" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="35" customHeight="1">
       <c r="A115" s="8" t="inlineStr">
@@ -8978,6 +9624,11 @@
         </is>
       </c>
       <c r="N115" s="8" t="inlineStr"/>
+      <c r="O115" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="35" customHeight="1">
       <c r="A116" s="7" t="inlineStr">
@@ -9042,6 +9693,11 @@
         </is>
       </c>
       <c r="N116" s="7" t="inlineStr"/>
+      <c r="O116" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="35" customHeight="1">
       <c r="A117" s="8" t="inlineStr">
@@ -9106,6 +9762,11 @@
         </is>
       </c>
       <c r="N117" s="8" t="inlineStr"/>
+      <c r="O117" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="35" customHeight="1">
       <c r="A118" s="7" t="inlineStr">
@@ -9166,6 +9827,11 @@
         </is>
       </c>
       <c r="N118" s="7" t="inlineStr"/>
+      <c r="O118" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="35" customHeight="1">
       <c r="A119" s="8" t="inlineStr">
@@ -9226,6 +9892,11 @@
         </is>
       </c>
       <c r="N119" s="8" t="inlineStr"/>
+      <c r="O119" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="35" customHeight="1">
       <c r="A120" s="7" t="inlineStr">
@@ -9286,6 +9957,11 @@
         </is>
       </c>
       <c r="N120" s="7" t="inlineStr"/>
+      <c r="O120" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="35" customHeight="1">
       <c r="A121" s="8" t="inlineStr">
@@ -9346,6 +10022,11 @@
         </is>
       </c>
       <c r="N121" s="8" t="inlineStr"/>
+      <c r="O121" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="35" customHeight="1">
       <c r="A122" s="7" t="inlineStr">
@@ -9406,6 +10087,11 @@
         </is>
       </c>
       <c r="N122" s="7" t="inlineStr"/>
+      <c r="O122" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="35" customHeight="1">
       <c r="A123" s="8" t="inlineStr">
@@ -9466,6 +10152,11 @@
         </is>
       </c>
       <c r="N123" s="8" t="inlineStr"/>
+      <c r="O123" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="35" customHeight="1">
       <c r="A124" s="7" t="inlineStr">
@@ -9526,6 +10217,11 @@
         </is>
       </c>
       <c r="N124" s="7" t="inlineStr"/>
+      <c r="O124" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="35" customHeight="1">
       <c r="A125" s="8" t="inlineStr">
@@ -9590,6 +10286,11 @@
         </is>
       </c>
       <c r="N125" s="8" t="inlineStr"/>
+      <c r="O125" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="35" customHeight="1">
       <c r="A126" s="7" t="inlineStr">
@@ -9654,6 +10355,11 @@
         </is>
       </c>
       <c r="N126" s="7" t="inlineStr"/>
+      <c r="O126" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="35" customHeight="1">
       <c r="A127" s="8" t="inlineStr">
@@ -9718,6 +10424,11 @@
         </is>
       </c>
       <c r="N127" s="8" t="inlineStr"/>
+      <c r="O127" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="35" customHeight="1">
       <c r="A128" s="7" t="inlineStr">
@@ -9782,6 +10493,11 @@
         </is>
       </c>
       <c r="N128" s="7" t="inlineStr"/>
+      <c r="O128" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="35" customHeight="1">
       <c r="A129" s="8" t="inlineStr">
@@ -9846,6 +10562,11 @@
         </is>
       </c>
       <c r="N129" s="8" t="inlineStr"/>
+      <c r="O129" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="35" customHeight="1">
       <c r="A130" s="7" t="inlineStr">
@@ -9910,6 +10631,11 @@
         </is>
       </c>
       <c r="N130" s="7" t="inlineStr"/>
+      <c r="O130" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="35" customHeight="1">
       <c r="A131" s="8" t="inlineStr">
@@ -9974,6 +10700,11 @@
         </is>
       </c>
       <c r="N131" s="8" t="inlineStr"/>
+      <c r="O131" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="35" customHeight="1">
       <c r="A132" s="7" t="inlineStr">
@@ -10038,6 +10769,11 @@
           <t>Rango: 0.0 – 1.0. Mayor = mayor prioridad de selección.</t>
         </is>
       </c>
+      <c r="O132" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="35" customHeight="1">
       <c r="A133" s="8" t="inlineStr">
@@ -10102,6 +10838,11 @@
           <t>Rango: 0.0 – 1.0. Mayor = mayor calidad del dato.</t>
         </is>
       </c>
+      <c r="O133" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="35" customHeight="1">
       <c r="A134" s="7" t="inlineStr">
@@ -10166,6 +10907,11 @@
           <t>Valores: ALTO, MEDIO, BAJO, CRITICO</t>
         </is>
       </c>
+      <c r="O134" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="35" customHeight="1">
       <c r="A135" s="8" t="inlineStr">
@@ -10230,6 +10976,11 @@
         </is>
       </c>
       <c r="N135" s="8" t="inlineStr"/>
+      <c r="O135" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="136" ht="35" customHeight="1">
       <c r="A136" s="7" t="inlineStr">
@@ -10294,6 +11045,11 @@
         </is>
       </c>
       <c r="N136" s="7" t="inlineStr"/>
+      <c r="O136" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="137" ht="35" customHeight="1">
       <c r="A137" s="8" t="inlineStr">
@@ -10358,6 +11114,11 @@
         </is>
       </c>
       <c r="N137" s="8" t="inlineStr"/>
+      <c r="O137" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="138" ht="35" customHeight="1">
       <c r="A138" s="7" t="inlineStr">
@@ -10422,6 +11183,11 @@
         </is>
       </c>
       <c r="N138" s="7" t="inlineStr"/>
+      <c r="O138" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="139" ht="35" customHeight="1">
       <c r="A139" s="8" t="inlineStr">
@@ -10486,6 +11252,11 @@
         </is>
       </c>
       <c r="N139" s="8" t="inlineStr"/>
+      <c r="O139" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="140" ht="35" customHeight="1">
       <c r="A140" s="7" t="inlineStr">
@@ -10546,6 +11317,11 @@
         </is>
       </c>
       <c r="N140" s="7" t="inlineStr"/>
+      <c r="O140" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="141" ht="35" customHeight="1">
       <c r="A141" s="8" t="inlineStr">
@@ -10606,6 +11382,11 @@
         </is>
       </c>
       <c r="N141" s="8" t="inlineStr"/>
+      <c r="O141" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="142" ht="35" customHeight="1">
       <c r="A142" s="7" t="inlineStr">
@@ -10666,6 +11447,11 @@
         </is>
       </c>
       <c r="N142" s="7" t="inlineStr"/>
+      <c r="O142" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="143" ht="35" customHeight="1">
       <c r="A143" s="8" t="inlineStr">
@@ -10726,6 +11512,11 @@
         </is>
       </c>
       <c r="N143" s="8" t="inlineStr"/>
+      <c r="O143" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="144" ht="35" customHeight="1">
       <c r="A144" s="7" t="inlineStr">
@@ -10786,6 +11577,11 @@
         </is>
       </c>
       <c r="N144" s="7" t="inlineStr"/>
+      <c r="O144" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="145" ht="35" customHeight="1">
       <c r="A145" s="8" t="inlineStr">
@@ -10850,6 +11646,11 @@
           <t>Puede ser igual al origen si no hubo transformación</t>
         </is>
       </c>
+      <c r="O145" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="146" ht="35" customHeight="1">
       <c r="A146" s="7" t="inlineStr">
@@ -10914,6 +11715,11 @@
           <t>Valores: EXITOSO, FALLIDO, OMITIDO</t>
         </is>
       </c>
+      <c r="O146" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="147" ht="35" customHeight="1">
       <c r="A147" s="8" t="inlineStr">
@@ -10974,6 +11780,11 @@
         </is>
       </c>
       <c r="N147" s="8" t="inlineStr"/>
+      <c r="O147" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="148" ht="35" customHeight="1">
       <c r="A148" s="7" t="inlineStr">
@@ -11038,6 +11849,11 @@
         </is>
       </c>
       <c r="N148" s="7" t="inlineStr"/>
+      <c r="O148" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="149" ht="35" customHeight="1">
       <c r="A149" s="8" t="inlineStr">
@@ -11098,6 +11914,11 @@
         </is>
       </c>
       <c r="N149" s="8" t="inlineStr"/>
+      <c r="O149" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="150" ht="35" customHeight="1">
       <c r="A150" s="7" t="inlineStr">
@@ -11158,6 +11979,11 @@
         </is>
       </c>
       <c r="N150" s="7" t="inlineStr"/>
+      <c r="O150" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="35" customHeight="1">
       <c r="A151" s="8" t="inlineStr">
@@ -11218,6 +12044,11 @@
         </is>
       </c>
       <c r="N151" s="8" t="inlineStr"/>
+      <c r="O151" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="152" ht="35" customHeight="1">
       <c r="A152" s="7" t="inlineStr">
@@ -11278,6 +12109,11 @@
         </is>
       </c>
       <c r="N152" s="7" t="inlineStr"/>
+      <c r="O152" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="153" ht="35" customHeight="1">
       <c r="A153" s="8" t="inlineStr">
@@ -11338,6 +12174,11 @@
         </is>
       </c>
       <c r="N153" s="8" t="inlineStr"/>
+      <c r="O153" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="154" ht="35" customHeight="1">
       <c r="A154" s="7" t="inlineStr">
@@ -11402,6 +12243,11 @@
           <t>Rango: 0.0 – 1.0</t>
         </is>
       </c>
+      <c r="O154" s="9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
     <row r="155" ht="35" customHeight="1">
       <c r="A155" s="8" t="inlineStr">
@@ -11466,6 +12312,11 @@
         </is>
       </c>
       <c r="N155" s="8" t="inlineStr"/>
+      <c r="O155" s="10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>